<commit_message>
Latest prices and website inputs
Uploading the latest prices and the input website list.
</commit_message>
<xml_diff>
--- a/websites.xlsx
+++ b/websites.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="41">
   <si>
     <t>URL</t>
   </si>
@@ -37,7 +37,7 @@
     <t>//*[@id="main"]/div/div/div[2]/div[2]/h1</t>
   </si>
   <si>
-    <t>//*[@id="main"]/div/div/div[2]/div[2]/p[1]</t>
+    <t>//*[@id="main"]/div/div/div[2]/div[2]/div[1]/p</t>
   </si>
   <si>
     <t>https://www.hy-vee.com/aisles-online/p/8657/Roma-Tomatoes</t>
@@ -49,6 +49,9 @@
     <t>https://www.hy-vee.com/aisles-online/p/3512698/Sara-Lee-Artesano-Brioche-Buns-8-count</t>
   </si>
   <si>
+    <t>//*[@id="main"]/div/div/div[2]/div[2]/div[1]/p[1]</t>
+  </si>
+  <si>
     <t>https://www.hy-vee.com/aisles-online/p/2886456/Thats-Smart-Mayonnaise</t>
   </si>
   <si>
@@ -73,6 +76,9 @@
     <t>https://www.hy-vee.com/aisles-online/p/371584/Wonderful-Halos-Mandarin-Oranges</t>
   </si>
   <si>
+    <t>//*[@id="main"]/div/div/div[1]/div[2]/div[1]/p</t>
+  </si>
+  <si>
     <t>https://www.hy-vee.com/aisles-online/p/31823/Certified-Ground-Round-90-Lean-10-Fat</t>
   </si>
   <si>
@@ -85,16 +91,16 @@
     <t>//*[@id="secondary_navigation"]/div/div/div/div[1]/div[1]/div/div[1]/div/div[3]</t>
   </si>
   <si>
-    <t>//*[@id="blurb_rail_copy_copy"]/div/div/div/div/div/div[1]/div/div/div[1]/div[2]/div[2]</t>
+    <t>//*[@id="blurb_rail_copy_copy"]/div/div/div/div/div/div[1]/div/div/div[1]/div[2]/div[1]</t>
   </si>
   <si>
     <t>https://www.chevrolet.com/trucks/silverado/1500</t>
   </si>
   <si>
-    <t>//*[@id="gb-main-content"]/div[1]/div[1]/gb-adv-grid/adv-col[1]/div/h1</t>
-  </si>
-  <si>
-    <t>//*[@id="gb-main-content"]/gb-adv-grid[2]/adv-col[2]/div/gb-adv-grid/adv-col[1]/div/div/div/p/span</t>
+    <t>//*[@id="gb-main-content"]/gb-adv-grid[1]/adv-col/div/div/div[1]/gb-adv-grid/adv-col[1]/div/h1</t>
+  </si>
+  <si>
+    <t>//*[@id="gb-main-content"]/gb-adv-grid[1]/adv-col/div/gb-adv-grid[3]/adv-col[1]/div/gb-adv-grid/adv-col[1]/div/div/div/p/span</t>
   </si>
   <si>
     <t>https://www.menards.com/main/building-materials/lumber-boards/dimensional-lumber/2-x-4-construction-framing-lumber/1021101/p-1444451086852-c-13125.htm</t>
@@ -118,17 +124,23 @@
     <t>//*[@id="root"]/div/div/div[5]/div[1]/div/div[3]/span/h1</t>
   </si>
   <si>
-    <t>//*[@id="eco-rebate-price"]/div/div[1]/div/div/span[2]</t>
+    <t>//*[@id="eco-rebate-price"]/div/div[1]/div/span[2]</t>
   </si>
   <si>
     <t>https://www.homedepot.com/p/Samsung-7-4-cu-ft-Vented-Smart-Front-Load-Electric-Dryer-with-Steam-Sanitize-in-White-DVE55CG7100W/325807880</t>
+  </si>
+  <si>
+    <t>//*[@id="root"]/div/div/div[5]/div/div[1]/div/div[3]/span/h1</t>
+  </si>
+  <si>
+    <t>https://www.hy-vee.com/aisles-online/p/3594226/Folgers-Coffee-Classic-Roast-Ground-Medium</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -139,6 +151,10 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="2">
@@ -155,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -163,6 +179,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -444,12 +463,12 @@
         <v>7</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>7</v>
@@ -460,7 +479,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>7</v>
@@ -471,7 +490,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>7</v>
@@ -482,7 +501,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>7</v>
@@ -493,7 +512,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>7</v>
@@ -504,7 +523,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>7</v>
@@ -515,7 +534,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>7</v>
@@ -526,18 +545,18 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>7</v>
@@ -548,7 +567,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>7</v>
@@ -559,40 +578,40 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>7</v>
@@ -603,7 +622,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>7</v>
@@ -614,27 +633,41 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="A24"/>
+  </hyperlinks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>